<commit_message>
Checkpoint 5 & Checkpoint 6
</commit_message>
<xml_diff>
--- a/数据表/Entity/Enemy.xlsx
+++ b/数据表/Entity/Enemy.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>#</t>
   </si>
@@ -49,6 +49,15 @@
     <t>HpAddPerLevel</t>
   </si>
   <si>
+    <t>AttackDamage</t>
+  </si>
+  <si>
+    <t>AttackCooldown</t>
+  </si>
+  <si>
+    <t>AttackRange</t>
+  </si>
+  <si>
     <t>Speed</t>
   </si>
   <si>
@@ -61,12 +70,18 @@
     <t>DropPercent</t>
   </si>
   <si>
+    <t>Params</t>
+  </si>
+  <si>
     <t>int</t>
   </si>
   <si>
     <t>float</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
     <t>敌人编号</t>
   </si>
   <si>
@@ -82,6 +97,15 @@
     <t>每关卡增加生命</t>
   </si>
   <si>
+    <t>基础伤害</t>
+  </si>
+  <si>
+    <t>攻击间隔</t>
+  </si>
+  <si>
+    <t>攻击范围</t>
+  </si>
+  <si>
     <t>移动速度</t>
   </si>
   <si>
@@ -94,7 +118,16 @@
     <t>掉落概率</t>
   </si>
   <si>
+    <t>额外参数</t>
+  </si>
+  <si>
     <t>近战敌人</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>远程敌人</t>
   </si>
 </sst>
 </file>
@@ -1028,21 +1061,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="4"/>
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
     <col min="2" max="2" width="18.7272727272727" style="1" customWidth="1"/>
     <col min="3" max="4" width="18.6363636363636" style="1" customWidth="1"/>
     <col min="5" max="5" width="19.4545454545455" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.0909090909091" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.2727272727273" style="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1818181818182" style="1" customWidth="1"/>
-    <col min="9" max="9" width="11.2727272727273" style="1" customWidth="1"/>
-    <col min="10" max="10" width="13.4545454545455" style="1" customWidth="1"/>
+    <col min="6" max="7" width="18.0909090909091" style="1" customWidth="1"/>
+    <col min="8" max="10" width="15.2727272727273" style="1" customWidth="1"/>
+    <col min="11" max="11" width="11.1818181818182" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.2727272727273" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13.4545454545455" style="1" customWidth="1"/>
+    <col min="14" max="14" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1050,7 +1084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:14">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1078,74 +1112,110 @@
       <c r="J2" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:14">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:14">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>20</v>
+        <v>25</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:14">
       <c r="B5" s="1">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="D5" s="1">
         <v>101</v>
@@ -1157,16 +1227,69 @@
         <v>50</v>
       </c>
       <c r="G5" s="1">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1</v>
+      </c>
+      <c r="I5" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="J5" s="1">
         <v>3</v>
       </c>
-      <c r="H5" s="1">
+      <c r="K5" s="1">
         <v>5</v>
       </c>
-      <c r="I5" s="1">
+      <c r="L5" s="1">
         <v>1</v>
       </c>
-      <c r="J5" s="1">
+      <c r="M5" s="1">
         <v>0.3</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="B6" s="1">
+        <v>2</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="1">
+        <v>102</v>
+      </c>
+      <c r="E6" s="1">
+        <v>40</v>
+      </c>
+      <c r="F6" s="1">
+        <v>40</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+      <c r="H6" s="1">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>8</v>
+      </c>
+      <c r="J6" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="K6" s="1">
+        <v>4</v>
+      </c>
+      <c r="L6" s="1">
+        <v>2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>